<commit_message>
App: on-phone mode (no account, offline), supplier orders, share plan, clearance floor price
- 'Start on this phone': every screen runs on the device with the shared engine
  (same results as the server), data saved in the app's private storage. AI features
  explain they need an account. Free/Pro can be switched in the test build.
- Supplier orders: what to reorder, grouped by supplier, with the order message
  written and sent through the phone's share sheet (WhatsApp, email, text)
- Weekly Plan: share button and a shortcut to supplier orders
- Clearing slow stock now names the lowest price that still covers cost and fees
  (backend and engine give identical plans)
- Engine decodes text without TextDecoder, so it runs the same on phones
- Sample stock lists include made-up suppliers
- preview/build_preview.py also refreshes the app's copy of the engine

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASabdzQTL4KaCGW6RUe1id
</commit_message>
<xml_diff>
--- a/stockpilot/docs/sample-data/my-shop-spreadsheet-sample.xlsx
+++ b/stockpilot/docs/sample-data/my-shop-spreadsheet-sample.xlsx
@@ -27900,7 +27900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27931,6 +27931,11 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Supplier days</t>
         </is>
       </c>
@@ -27955,7 +27960,12 @@
       <c r="E2" t="n">
         <v>13.5</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>EcoPet Supply</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
         <v>14</v>
       </c>
     </row>
@@ -27979,7 +27989,12 @@
       <c r="E3" t="n">
         <v>22</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Green Paws Trading</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
         <v>21</v>
       </c>
     </row>
@@ -28003,7 +28018,12 @@
       <c r="E4" t="n">
         <v>11</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>EcoPet Supply</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
         <v>14</v>
       </c>
     </row>
@@ -28027,7 +28047,12 @@
       <c r="E5" t="n">
         <v>35</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Green Paws Trading</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
         <v>28</v>
       </c>
     </row>
@@ -28051,7 +28076,12 @@
       <c r="E6" t="n">
         <v>15</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>EcoPet Supply</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
         <v>14</v>
       </c>
     </row>

</xml_diff>